<commit_message>
saw an error with one of the analyses and fixed it
</commit_message>
<xml_diff>
--- a/data/humanEBBinom.xlsx
+++ b/data/humanEBBinom.xlsx
@@ -413,191 +413,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Parent EB vs Daughter EB</t>
+        </is>
+      </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Parent EB</t>
+          <t>Mouse EB vs Parent EB</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Human EB</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Human EB</t>
+          <t>Mouse EB vs Daughter EB</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Daughter EB</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>numAboveLine</t>
-        </is>
+          <t>numAboveLine (Y&gt;X)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>38</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>numBelowLine</t>
-        </is>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>numBelowLine (Y&lt;X)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>13</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>totalNum</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>43</v>
+      </c>
       <c r="C4" t="n">
-        <v>65</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+        <v>43</v>
+      </c>
+      <c r="D4" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>pValue</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>0.004077315330505371</v>
+      </c>
       <c r="C5" t="n">
-        <v>0.0006210434562277101</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Parent EB</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>numAboveLine</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="n">
-        <v>29</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>numBelowLine</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="n">
-        <v>7</v>
-      </c>
-      <c r="E7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>totalNum</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="n">
-        <v>65</v>
-      </c>
-      <c r="E8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>pValue</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="n">
-        <v>0.0003125511575490236</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Daughter EB</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>numAboveLine</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="n">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>numBelowLine</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>totalNum</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="n">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>pValue</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="n">
-        <v>1.308758612594829e-08</v>
+        <v>0.6476058959960938</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.005222879350185395</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A6:A9"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>